<commit_message>
Separar Primer Nivel / Segundo Nivel en columnas propias (antes iban combinados en una sola celda)
Confirmado en vivo que 'Cortes Y Reposicion Del Servicio' es un 2do nivel
real bajo Comercial (con 4 pantallas aun sin automatizar: Solicitud/Emision
De Ordenes Especiales De Corte y Reconexion), lo que expuso que mezclar
ambos niveles en una celda de texto ocultaba la jerarquia real.
</commit_message>
<xml_diff>
--- a/Opciones_Menu_Principal.xlsx
+++ b/Opciones_Menu_Principal.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Opciones de Menu" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opciones de Menu'!$A$1:$D$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Opciones de Menu'!$A$1:$E$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,32 +431,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Categoria (1er nivel - 2do nivel)</t>
+          <t>Primer Nivel</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Segundo Nivel</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Opcion del menu</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>RF</t>
         </is>
@@ -468,17 +474,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Administración De Planes De Encargo</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -490,17 +497,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Administración De Tipos De Cambio</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -512,17 +520,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Afiliaciones Por Promotores Especiales</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
@@ -534,17 +543,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Anulacion De Facturas</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -556,17 +566,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Aprobación De Informes Dwh</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>RF-10</t>
         </is>
@@ -578,17 +589,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Asignacion De Clientes A Carteras</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -600,17 +612,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Auditoria De Afiliaciones</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -622,17 +635,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Cambio De Estado De Libros De Corte</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP4</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -644,17 +658,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Comisión De Encargos De Cobranza</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
@@ -666,17 +681,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Consulta De Catastro De Conexiones Eléctricas</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
@@ -688,17 +704,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Consulta De Clientes Asociados A Una S.S.</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP2</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -710,17 +727,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Consulta De Cortes Pendientes</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP2</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
@@ -732,17 +750,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Consulta De Cuadratura De Sesion</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP2</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -754,17 +773,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Consulta De Movimientos De Saldos</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
@@ -776,17 +796,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Consulta De Proyectos De Encargos</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -798,17 +819,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Consulta Generica De Solicitudes De Reposicion</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP2</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>RF-09</t>
         </is>
@@ -820,17 +842,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Emisión De Cartas Masivas</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
@@ -842,17 +865,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Encargos De Cobranza</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
@@ -864,17 +888,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Ingreso De Accion Realizada - Ordenes Especiales De Corte</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP4</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -886,17 +911,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Ingreso De Accion Realizada Para Ordenes De Reposicion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP4</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -908,17 +934,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Ingreso De Libros De Corte</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP4</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -930,17 +957,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Investigacion De Clientes</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -952,17 +980,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Listados De Corte Y Reposicion</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP4</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
@@ -974,17 +1003,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Listados De Facilidades De Pago Por Deuda De Energía</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
@@ -996,17 +1026,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Listados De Ingresos De Cnr Por Deuda De Servicios</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>RF-09</t>
         </is>
@@ -1018,17 +1049,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Log De Carga De Datawarehouse</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
@@ -1040,17 +1072,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Mantenedor De Inspectores De Corte</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP2</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -1062,17 +1095,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Mantenimiento De Carteras</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -1084,17 +1118,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Mantenimiento De Clientes De Encargos</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -1106,17 +1141,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Mantenimiento De Informes Dwh</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>RF-11</t>
         </is>
@@ -1128,17 +1164,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Mantenimiento De Promotores</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -1150,17 +1187,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Mantenimiento De Seguros De Encargo</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -1172,17 +1210,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Niveles De Promotor</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
@@ -1194,17 +1233,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Parámetros De Encargo</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP6</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -1216,17 +1256,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Promocion De Afiliados</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -1238,17 +1279,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Restaura Y Transfiere A Proceso</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -1260,17 +1302,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Resumen De Afiliacion</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP7</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
@@ -1282,17 +1325,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Seleccion De Clientes Afectos A Corte</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP4</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -1304,17 +1348,18 @@
           <t>Comercial</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Traslado De Clientes</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>PR000349-SP1</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>RF-01, RF-03</t>
         </is>
@@ -1323,20 +1368,25 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Atención Integral Al Cliente</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
+          <t>Atención Integral Al Cliente</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
           <t>Asignacion De Usuarios</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>PR000335-SP5</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -1345,20 +1395,25 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Atención Integral Al Cliente</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
+          <t>Atención Integral Al Cliente</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
           <t>Atenciones A Clientes &gt; Consulta De Atenciones Comerciales</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>PR000335-SP2</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>RF-01, RF-02, RF-03, RF-04</t>
         </is>
@@ -1367,20 +1422,25 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Atención Integral Al Cliente</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>Atención Integral Al Cliente</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>Atenciones A Clientes &gt; Consulta De Atenciones Comerciales</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>PR000335-SP4</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>RF-01, RF-03</t>
         </is>
@@ -1389,20 +1449,25 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Atención Integral Al Cliente</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
+          <t>Atención Integral Al Cliente</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>Listado Pedidos Importantes</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>PR000335-SP5</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -1411,20 +1476,25 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Atención Integral Al Cliente</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
+          <t>Atención Integral Al Cliente</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
           <t>Resumen De Pedidos</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>PR000335-SP5</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -1433,20 +1503,25 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Atención Integral Al Cliente</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
+          <t>Atención Integral Al Cliente</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
           <t>Seguimiento De Clientes Mt</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>PR000335-SP5</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -1455,20 +1530,25 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Facturación</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
+          <t>Facturación</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
           <t>Refacturación &gt; Traslados De Capital - Órdenes De Refacturación</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP6</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>RF-01, RF-02, RF-03, RF-04, RF-05, RF-06, RF-07, RF-08, RF-09, RF-10</t>
         </is>
@@ -1477,20 +1557,25 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
           <t>Acuerdos Del Reclamo</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
@@ -1499,20 +1584,25 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
           <t>Asignacion De Reclamos</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>RF-02, RF-09</t>
         </is>
@@ -1521,20 +1611,25 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
           <t>Atención Rápida - Conciliación De Tres Dias</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -1543,20 +1638,25 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
           <t>Búsqueda De Reclamos</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>RF-05, RF-06</t>
         </is>
@@ -1565,20 +1665,25 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
           <t>Cargo De Recepcion Osinerg</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
@@ -1587,20 +1692,25 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
           <t>Consulta Detalle Reclamo</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -1609,20 +1719,25 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
           <t>Mantenedor Gestión Reclamo</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -1631,20 +1746,25 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
           <t>Mis Reclamos</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -1653,20 +1773,25 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Comercial - Reclamos Comerciales</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
+          <t>Reclamos Comerciales</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
           <t>Reasignación De Reclamos</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>PR000326-SP2</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>RF-03, RF-06, RF-09</t>
         </is>
@@ -1678,17 +1803,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Actualización De Agenda De Facturación</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>RF-10</t>
         </is>
@@ -1700,17 +1826,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Actualización De Agenda De Pagos</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -1722,17 +1849,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Actualización De Conceptos</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
@@ -1744,17 +1872,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Actualización De Documentos</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -1766,17 +1895,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Actualización De Oficinas De La Cia</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP4</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>RF-01, RF-03, RF-05, RF-06, RF-07, RF-08, RF-11</t>
         </is>
@@ -1788,17 +1918,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Actualización De Precios</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
@@ -1810,17 +1941,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Actualización De Tasas De Interés</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
@@ -1832,17 +1964,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Mantenedor De Tablas Del Sistema Comercial</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
@@ -1854,17 +1987,18 @@
           <t>Interno</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr"/>
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Relación Sucursal - Sector - Zona</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP3</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -1873,20 +2007,25 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Interno - Plataforma Web</t>
+          <t>Interno</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
+          <t>Plataforma Web</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
           <t>Consulta De Lecturas De Maxímetro</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP7</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
@@ -1895,20 +2034,25 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Interno - Plataforma Web</t>
+          <t>Interno</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>Plataforma Web</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
           <t>Corrección De Demandas Leídas Históricas</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP7</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
@@ -1917,20 +2061,25 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Interno - Plataforma Web</t>
+          <t>Interno</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>Plataforma Web</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
           <t>Corrección De Lecturas De Facturación</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP7</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
@@ -1939,20 +2088,25 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Interno - Plataforma Web</t>
+          <t>Interno</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
+          <t>Plataforma Web</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
           <t>Corrección De Lecturas Maxímetros</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP7</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
@@ -1961,27 +2115,32 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Interno - Plataforma Web</t>
+          <t>Interno</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
+          <t>Plataforma Web</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
           <t>Corrección De Lecturas Ordinarias</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>PR000325-SP7</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D70"/>
+  <autoFilter ref="A1:E70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>